<commit_message>
fix: 코딩 모드 Phase 1 게이트 - Claude 코드 완성 전 Codex/Gemini 자동 진입 차단 (v0.6.4)
Claude 가 요구사항을 되묻는 질문 응답을 줬을 때 봇이 그것을 코드로 간주하여
Phase 2 Codex 리뷰가 곧장 시작되고 stockradar stacktrace 같은 엉뚱한 컨텍스트를
끌어와 응답하던 회귀를 수정. Phase 3 Gemini 응답 없음 문제도 함께 해결.

- AWAIT_USER 태그 + 모듈 전역 pending dict + threading lock 으로 Phase 1 게이트
- start/_resume_pending 에 inflight guard, fenced code block 오탐 차단,
  UUID sentinel, image 병합 dedup, cancel pending 정리 포함
- 단위 테스트 23건 추가 (전체 61 passed)
- Codex 교차 검증 3차 라운드 (race/cancel/fenced/image/placeholder 이슈 반영)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5457,6 +5457,71 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>코딩 모드 Phase 1 게이트: Claude 코드 완성 전 Codex/Gemini 자동 진입 차단</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>코딩 모드 사용 (CODING_CHANNEL_ID 채널), Phase 1 Claude 응답에 코드 없이 사용자에게 되묻는 질문만 있는 경우</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1. 코딩 채널에 모호한 요청 (예: "커플 웹사이트 만들고 싶어 기획부터")
+2. Phase 1 Claude 가 요구사항 질문으로 응답
+3. 봇이 Claude 응답을 코드로 간주하여 Phase 2 Codex 리뷰 즉시 시작
+4. Codex 가 엉뚱한 stockradar stacktrace 컨텍스트 출력 (277초)
+5. Phase 3 Gemini 는 도달도 못 하고 응답 없음</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>원인: modes/coding.py start() 가 Phase 1 → 2 → 3 무조건 순차 진행. Claude 가 코드 대신 질문으로 응답할 수 있다는 케이스 미처리.
+수정: AWAIT_USER_PATTERN 태그 + 모듈 전역 _PENDING_THREADS dict + threading.Lock + _INFLIGHT_PHASE1 set 으로 Phase 1 게이트 도입. start() 가 태그 감지 시 pending 등록 후 Phase 2/3 호출 없이 종료. followup 에서 사용자 답변 받아 Claude 재호출, 응답에 태그 사라지면 _run_review_and_test() 자동 호출. fenced code block 오탐 방지, UUID sentinel, image 병합 dedup, cancel pending 정리 포함.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>CodingMode (start/followup) - 모호한 요구사항 + 이미지 첨부 + 동시 followup 시나리오 전반</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>v0.6.3</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>v0.6.4</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: v0.7.5 회귀 핫픽스 - slack_bot.py 의 os import 누락 (v0.7.6)
v0.7.5 commit (a37ae5f) 직후 실전 PDF 첨부 테스트에서 봇 완전 무응답.
bot_output.log 의 NameError 로 진단:

  Exception in thread Thread-10 (_runner):
  File "slack_bot.py", line 173, in _runner
    base_tmp = os.path.join(os.path.dirname(os.path.abspath(__file__)), ".tmp")
  NameError: name 'os' is not defined

원인: v0.7.5 에서 tmp_dir 을 <project>/.tmp/ 내부로 옮길 때 _runner 안에서
os.path.join / os.makedirs 를 추가했는데 모듈 전역에 import os 가 없음.
함수 내부 import tempfile, shutil 만 추가하고 os 는 빠뜨림.

수정:
- slack_bot.py 모듈 전역 import 에 os 추가
- tests/test_slack_bot.py 에 test_os_module_imported 회귀 테스트 추가

영향:
- v0.7.5 commit 부터 v0.7.6 fix 까지 약 30분간 PDF/이미지 첨부 무응답
- 첨부 없는 텍스트 메시지는 정상 (라우팅이 _runner 진입 전 분기)

검증:
- pytest tests/test_slack_bot.py 11 passed (기존 10 + 신규 1)
- python -c "import slack_bot" 통과

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6371,6 +6371,69 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>v0.7.5 자체 회귀: slack_bot.py 의 os import 누락으로 PDF/이미지 첨부 시 _runner NameError 무응답</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>v0.7.5 (a37ae5f) 배포 직후 실전 PDF 첨부 테스트 (슬랙 스레드 1779797934.173099)</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>1. v0.7.5 봇 재시작 후 슬랙 채널에 PDF 첨부 + 평가 요청 메시지
+2. 봇 완전 무응답 (Round 1/2/3 진행 표시조차 없음)
+3. bot_output.log 확인: Exception in thread Thread-10 (_runner): NameError: name 'os' is not defined (slack_bot.py:173)
+4. 첨부 없는 일반 텍스트 메시지는 정상 동작 (라우팅이 _runner 진입 전 분기)</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>원인: v0.7.5 에서 tmp_dir 을 &lt;project&gt;/.tmp/ 내부로 옮길 때 _runner 안에서 os.path.join / os.makedirs 를 추가했는데 모듈 전역에 import os 가 없음. 함수 내부 import tempfile, shutil 만 추가하고 os 는 빠뜨림. 수정: (A) slack_bot.py 모듈 전역 import 에 os 추가. (B) tests/test_slack_bot.py 에 test_os_module_imported 회귀 테스트 추가 (모듈에 os attribute 존재 + 진짜 os 모듈인지 검증).</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>slack_bot.py + tests/test_slack_bot.py. v0.7.5 commit 부터 v0.7.6 fix 까지 약 30분간 모든 첨부 메시지 봇 무응답.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>v0.7.5</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>v0.7.6</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Gemini "True color (24-bit) support not detected" 터미널 경고 누출 수정 (v0.7.8)
non-TTY 환경에서 Gemini CLI 가 매 호출 첫 줄에 찍는 색상 경고가
Slack 답변 본문 앞에 노출됨 (자체 테스트 thread 1780059304 에서 발견).

원인: agents/gemini.py 의 _clean_output 노이즈 필터가 _NOISE_KEYWORDS
포함 라인을 제거하는데, 색상 경고로 "256-color support not detected" 만
등록돼 있어 실제 출력되는 "True color (24-bit) support not detected"
변종이 통과해 응답에 섞임.

- agents/gemini.py: _NOISE_KEYWORDS 의 "256-color support not detected" 를
  공통 꼬리 "support not detected" 로 교체 (256-color/True color 변종 모두 필터).
- tests/test_gemini.py: true-color 24-bit 경고 회귀 테스트 추가.
- 단위 269 passed, 실제 Gemini 호출 + 슬랙 전수 스캔(모든 발언) 누출 0건,
  Codex 교차검증 통과.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6496,6 +6496,67 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Gemini 매 발언 첫 줄에 'True color (24-bit) support not detected' 터미널 경고 누출</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>non-TTY 환경에서 Gemini CLI 호출 시 (자체 테스트 thread 1780059304.126349)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>1. stockradar 채널에서 토론 실행
+2. Gemini 발언마다 첫 줄에 'Warning: True color (24-bit) support not detected. Using a terminal with true color enabled will result in a better visual experience.' 가 본문 앞에 노출됨</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>원인: agents/gemini.py 의 _clean_output 노이즈 필터가 _NOISE_KEYWORDS 의 키워드 포함 라인을 제거하는데, 색상 경고로 '256-color support not detected' 만 등록돼 있어 실제 출력되는 'True color (24-bit) support not detected' 변종이 필터를 통과해 응답에 섞임. 수정: _NOISE_KEYWORDS 의 '256-color support not detected' 를 공통 꼬리 'support not detected' 로 교체하여 256-color/True color(24-bit) 및 향후 변종을 모두 필터. tests/test_gemini.py::TestCleanOutput 에 true-color 케이스 회귀 테스트 추가. 단위 269 passed, 실제 Gemini 호출 + 슬랙 전수 스캔 확인, Codex 교차검증 통과. 추가: 자체 테스트가 합의문만 검사해 이 노이즈를 놓쳤던 문제도 전수 스캔 방식으로 개선.</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Gemini 에이전트 Slack 답변 외관. 기능 오류는 아니나 매 발언에 경고 노이즈 노출.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>v0.7.7</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>v0.7.8</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(gemini): agy -p stdout 버그(#76) 우회 - 디스크 transcript trace 토큰 복구
agy `--print`/`-p` 가 non-TTY(subprocess)에서 모델 응답을 stdout 에 안 쓰는
upstream 버그(google-antigravity/antigravity-cli#76, 2026-06-09 OPEN, 1.0.6
미수정)를 우회. 호출별 고유 trace 토큰을 prompt 끝에 심고, 디스크 transcript
(brain/<cid>/.../transcript.jsonl)의 그 토큰이 박힌 턴 응답을 회수한다. Gemini
CLI 개인 티어 2026-06-18 종료 대비 agy 백엔드 실사용 준비(v0.7.10).

- agents/gemini.py: _recover_agy_response/_extract_traced_response/_iter_turns
  /_trace_in 신설 + _run_cli/_run_progress_once 통합. cwd->cid 매핑 1차 +
  since_ts 스캔 2차(둘 다 토큰 매칭, 동시호출/대화재사용/공통prefix 오회수 방지).
- 보안: cid UUID 검증(_valid_cid)으로 path traversal 차단, content 정규화, 마커 strip.
- 검증: 라이브 실측 3회(stdin=DEVNULL, agy 1.0.6 EXIT=0/STDOUT_LEN=0 인데 토큰
  복구로 정확 회수) + 단위 테스트 22건 신규 + Codex 3차 교차검증 통과.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6619,6 +6619,62 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>agy `-p` stdout 미출력 버그(#76) 우회 - 디스크 transcript 에서 trace 토큰으로 응답 복구</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>agy(Antigravity CLI) 백엔드(GEMINI_CLI_BINARY=agy)에서 `-p`가 non-TTY 에 stdout 응답을 안 쓰는 upstream 버그(#76)를 우회. 호출별 고유 trace 토큰(AGYTRACE+uuid)을 prompt 끝에 심고(argv 절단 이후 append 로 유실 방지), 디스크 transcript (brain/&lt;cid&gt;/.system_generated/logs/transcript.jsonl)의 USER_INPUT 에서 그 토큰이 박힌 턴의 최종 PLANNER_RESPONSE 만 회수. _recover_agy_response/_extract_traced_response/_iter_turns/_trace_in 신설, _run_cli·_run_progress_once 통합. cwd→cid 매핑 1차 + since_ts 이후 transcript 스캔 2차(둘 다 토큰 매칭). cid UUID 검증·content 정규화·마커 strip 포함.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Gemini CLI 개인 티어가 2026-06-18 종료 예정인데, 후계 agy 는 #76(2026-06-09 OPEN, 1.0.6 미수정)으로 비대화형 stdout 이 비어 봇 백엔드로 못 썼다. 응답이 디스크엔 정상 저장되는 점을 이용해 복구 경로를 붙여 agy 를 실사용 가능 상태로 준비. trace 토큰 방식이라 동시 호출/대화 재사용/공통 prompt prefix 에도 다른 호출 응답을 오회수하지 않음. Codex 3차 교차검증 통과 + 라이브 실측 3회(stdin=DEVNULL 에서 agy 1.0.6 EXIT=0/STDOUT_LEN=0 인데 토큰 복구로 정확 회수).</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>agents/gemini.py (GEMINI_CLI_BINARY=agy 경로). gemini 기본 경로는 토큰 무시로 무영향.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>v0.7.9</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>v0.7.10</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Windows에서 claude 호출 시 전역 MCP(context7 npx) spawn 으로 인한 cmd 창 깜빡임 제거 (v0.7.11)
원인: 봇이 `cmd /c claude -p` 로 호출하면 claude 가 부팅하며 사용자 전역 MCP
context7(npx -y @upstash/context7-mcp, stdio)을 `cmd /c npx` 로 새로 spawn.
claude.exe 가 CREATE_NO_WINDOW(숨김 콘솔)로 떠 있어 이 손자 프로세스가 부모의
숨김 콘솔을 못 물려받고 새 conhost 콘솔을 할당 → 잠깐 떴다 사라지는 깜빡임.

수정: claude 호출(_build_cmd/_build_stream_cmd/bridge _call_claude)에
--strict-mcp-config 추가 → 전역 MCP 0개 로드. 봇 답변은 빌트인 WebSearch/
WebFetch/Read 만 쓰므로 기능 영향 없음. codex(MCP url= HTTP 원격)·gemini 무관.

검증: 격리 PID 서브트리 실측(있음 spawn=False / 없음 spawn=True) + 단위
테스트(순서 단언 포함) + Codex 교차검증 통과(이슈 2건 모두 Trivial, 보강 완료).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6638,7 +6638,6 @@
           <t>agy `-p` stdout 미출력 버그(#76) 우회 - 디스크 transcript 에서 trace 토큰으로 응답 복구</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>agy(Antigravity CLI) 백엔드(GEMINI_CLI_BINARY=agy)에서 `-p`가 non-TTY 에 stdout 응답을 안 쓰는 upstream 버그(#76)를 우회. 호출별 고유 trace 토큰(AGYTRACE+uuid)을 prompt 끝에 심고(argv 절단 이후 append 로 유실 방지), 디스크 transcript (brain/&lt;cid&gt;/.system_generated/logs/transcript.jsonl)의 USER_INPUT 에서 그 토큰이 박힌 턴의 최종 PLANNER_RESPONSE 만 회수. _recover_agy_response/_extract_traced_response/_iter_turns/_trace_in 신설, _run_cli·_run_progress_once 통합. cwd→cid 매핑 1차 + since_ts 이후 transcript 스캔 2차(둘 다 토큰 매칭). cid UUID 검증·content 정규화·마커 strip 포함.</t>
@@ -6672,6 +6671,66 @@
       <c r="L106" t="inlineStr">
         <is>
           <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Windows 슬랙 문의 시 cmd 콘솔 창 깜빡임 (claude 호출의 전역 MCP context7 spawn)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>사용자 전역 Claude 설정에 stdio 방식 MCP(context7 = npx -y @upstash/context7-mcp) 등록 + Windows 환경</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>슬랙에서 봇에 문의 → 에이전트 '생각 중' 진입 시점에 cmd/conhost 콘솔 창이 잠깐 떴다 사라짐. claude 에이전트가 호출될 때마다 재현(가끔처럼 보이나 claude 경로면 상시).</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>원인: 봇이 `cmd /c claude -p ...` 로 Claude Code CLI 호출 시, claude 가 부팅하며 전역 MCP context7 을 `cmd /c npx ...` 로 새로 spawn. claude.exe 가 CREATE_NO_WINDOW(숨김 콘솔)로 떠 있어 이 손자 프로세스가 부모 숨김 콘솔을 못 물려받고 새 conhost 콘솔을 할당 → 깜빡임. 수정: claude 호출부(agents/claude.py _build_cmd/_build_stream_cmd, modes/bridge.py _call_claude)에 `--strict-mcp-config` 추가 → 전역 MCP 0개 로드(context7 spawn 제거). 라이브 격리 비교(있음 spawn=False / 없음 spawn=True) + Codex 교차검증 통과.</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>agents/claude.py, modes/bridge.py. Windows 에서 claude 에이전트가 타는 모든 경로(토론/브릿지/첨부 분석). codex(MCP url= HTTP 원격)·gemini 무관.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>v0.7.10</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>v0.7.11</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Minor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(research): v0.8.0 릴리즈 노트 + 이슈 로그(#107 enhancement)
리서치 모드 신설 기록. RELEASE_NOTES v0.8.0 섹션(배경/기능/검증) +
issue_log 107행(enhancement/Major, 발생 v0.7.11 → 수정 v0.8.0).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6734,6 +6734,62 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>리서치 모드 신설 (#ai-리서치, 3 AI 분담형 팬아웃 조사+교차검증+출처 리포트)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>#ai-리서치 채널 질문 → 분해(claude, 하위질문 JSON) → 하위질문 라운드로빈 분담 조사(claude/codex/gemini 병렬, 웹) → 생산자!=검증자 교차검증(supported/disputed/unverified) → claude 종합 → Slack 스레드 전송. modes/research.py 신설(순수 엔진 함수 + ResearchMode), config(RESEARCH_CHANNEL_ID/RESEARCH_SUBQ_MAX)·slack_bot 라우팅. 견고성: 분해 실패 단일질문 degrade, asyncio.gather(return_exceptions=True), _ask_named 백업 인계, disputed/unverified 드롭 없이 리포트 표기.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>기능 확장 방향으로 토론 고도화+리서치를 원했고 둘이 같은 '근거 기반 협업 코어'(웹 근거·상호 교차검증·출처)를 공유 → 엔진 한 번 구현해 두 모드로 노출(Phase 1=리서치, Phase 2=토론 고도화). 실사용 가치(출처 달린 신뢰 리포트) + 토론 고도화 토대 확보.</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>modes/research.py(신규), config.py, slack_bot.py, README/.env.example. 신규 #ai-리서치 채널. 기존 토론/코딩/브릿지 모드 무영향.</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>v0.7.11</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>v0.8.0</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(watchdog): !bot restart 1회에 봇 5중 spawn 수정 + 단일 인스턴스 lock 하드닝 (v0.8.9)
원인: 단일 인스턴스/단일 스레드 워치독인데도 start_bot() 재진입 가드가 비원자적(TOCTOU)
이라 재시작이 짧게 겹치면 봇이 중복 spawn.

- restart_bot: 재진입 가드(_restart_in_progress) + 디바운스(RESTART_DEBOUNCE=10s, monotonic)
  로 단일 명령=단일 재시작 보장. finally 에서 auto_restart/manual_stop/_restart_in_progress
  를 항상 정상 복구(예외 시 플래그 누수 차단)
- 단일 인스턴스 lock 을 Windows named mutex(CreateMutexW, 원자적·종료 시 OS 자동 해제)로
  전환 -> stale/빈창/double-takeover race 원천 소거, 생성 실패 시 fail-closed.
  비-Windows 폴백 파일락도 takeover 없이 fail-closed
- 신규/강화 test_watchdog 17건, 전체 405 통과
- Codex 교차검증 5라운드 전부 반영(Major 4 + Minor 4). 6라운드 확인은 컴패니언 작업
  정지로 보류, 마지막 auto_restart 수정은 직전 라운드 승인 패턴 + 테스트 커버

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7602,6 +7602,66 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>!bot restart 1회에 봇이 5중 spawn (재시작 재진입/중복)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>워치독 가동 중 Slack 명령 채널에서 !bot restart 전송</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>1. Slack 워치독 채널에 !bot restart 1회 전송 2. 워치독이 봇을 5개(서로 다른 PID, 일부 6ms 간격 동시) spawn 하고 '재시작 완료'를 5번 방송 3. 중복 봇은 Slack 소켓 충돌로 곧 죽고 1개로 수렴(증상은 일시적)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>원인: 워치독은 단일 인스턴스(.watchdog.lock)·단일 스레드인데도 start_bot() 의 재진입 가드(bot_process.poll() is None)가 비원자적(TOCTOU)이라 재시작이 짧게 겹치면 중복 spawn. 수정: restart_bot 에 재진입 가드(_restart_in_progress) + 디바운스(RESTART_DEBOUNCE=10s, monotonic)로 단일 명령=단일 재시작 보장. finally 에서 auto_restart/manual_stop/_restart_in_progress 를 항상 정상 복구(예외 시 플래그 누수로 크래시 자동재시작 건너뛰던 결함도 차단). 하드닝: 단일 인스턴스 lock 을 Windows named mutex(CreateMutexW, 원자적·종료 시 자동 해제)로 전환해 중복 워치독/stale/빈창/double-takeover race 원천 소거(생성 실패 시 fail-closed). 비-Windows 폴백도 takeover 없이 fail-closed. 신규/강화 테스트 17건, 전체 405 통과. Codex 교차검증 5라운드 전부 반영(Major 4 + Minor 4), 6라운드 확인은 컴패니언 작업 정지로 보류.</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>워치독 봇 재시작/단일 인스턴스 보장, Slack 명령 안정성</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>v0.8.8</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>v0.8.9</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(watchdog): mutex 전환 후 guard churn 방지 - lockfile PID heartbeat (v0.8.10)
v0.8.9 의 named mutex 전환으로 lockfile 을 안 쓰게 되자, watchdog_guard(3분 주기)의
lockfile 기반 생존체크가 'dead' 로 오판해 매 주기 헛 재기동(mutex ALREADY_EXISTS 로 즉시
종료)하던 churn 을 해소.

- acquire_lock(win32): mutex 획득 성공 후 .watchdog.lock 에 PID 를 heartbeat 로 기록.
  단일 인스턴스 보장은 여전히 mutex, lockfile 은 가드 정보용(race 무관).
- test_watchdog 17건(heartbeat 기록 단언, 실제 lockfile 미오염) + 전체 405 통과
- Codex 교차검증 핵심 4항목 통과(잔여 Minor 는 기존 가드 liveness 한계로 무관)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7662,6 +7662,66 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>mutex 전환 후 watchdog_guard 가 3분마다 헛 재기동(churn)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>v0.8.9 named mutex 전환(lockfile 미사용) + watchdog_guard 예약작업(3분 주기) 가동</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>1. 새 워치독이 단일 인스턴스를 mutex 로만 보장하고 .watchdog.lock 을 쓰지 않음 2. watchdog_guard.is_watchdog_running()이 .watchdog.lock 의 PID 로 생존 판정 -&gt; 'dead' 오판 3. 3분마다 워치독 재기동 시도 -&gt; 매번 mutex ERROR_ALREADY_EXISTS 로 즉시 종료(churn/콘솔깜빡임)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>원인: mutex 전환으로 lockfile 쓰기를 없앴는데 가드의 생존체크는 lockfile PID 기반이라 불일치. 수정: acquire_lock 의 Windows 경로에서 mutex 획득 성공 후 .watchdog.lock 에 PID 를 heartbeat 로 기록. 단일 인스턴스 보장은 여전히 mutex(원자적). lockfile 은 가드 정보용이라 race 무관. 가드가 live PID 를 보는 동안 lockfile 미변경 -&gt; 1회 기록으로 churn 해소. 종료/크래시 시 stale -&gt; 가드 정상 재기동. Codex 교차검증 핵심 4항목 통과(잔여 Minor 는 기존 가드 liveness 한계로 무관). test_watchdog 17건+전체 405 통과.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>워치독 가드 재기동 동작, 콘솔 깜빡임/리소스</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>v0.8.9</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>v0.8.10</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(gemini): TestBinarySelection 의 dev .env 누수 차단 - load_dotenv 무력화 (v0.8.12)
config.py 는 import 시 load_dotenv(override=True) 로 .env 를 읽는다.
TestBinarySelection 은 GEMINI_CLI_BINARY 를 monkeypatch 한 뒤
importlib.reload(config) 하는데, reload 가 load_dotenv(override=True) 를
재실행하며 dev .env 의 GEMINI_CLI_BINARY=agy(봇 실가동 설정)가 monkeypatch
값을 덮어써 default/empty/explicit-gemini/invalid 4건이 agy 로 잡혀 실패했다.

- tests/test_gemini.py: _restore_gemini_default autouse fixture 에
  monkeypatch.setattr("dotenv.load_dotenv", no-op) 추가. reload 가 .env 를
  다시 읽지 않아 monkeypatch 값이 유지됨. monkeypatch 가 teardown 이후 undo
  되므로 teardown reload 동안에도 패치 유효(gemini 기본값 정상 복원).
- production config.py 의 override=True(shell env 보다 .env 우선)는 봇
  동작상 의도된 정책이라 미변경.

TestBinarySelection 10건 통과(4실패->0), 전체 421건 통과. Codex 교차검증 통과.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7782,6 +7782,66 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>TestBinarySelection 4건이 dev .env 의 GEMINI_CLI_BINARY=agy 누수로 실패 (테스트 격리)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>로컬 .env 에 GEMINI_CLI_BINARY=agy 설정(봇 agy 실가동) 상태</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>1. .env 에 GEMINI_CLI_BINARY=agy 존재 2. pytest tests/test_gemini.py::TestBinarySelection 실행 3. default/empty/explicit-gemini/invalid 4건이 전부 agy 로 잡혀 실패 (agy 케이스만 우연히 .env 값과 일치해 통과)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>원인: config.py 가 import 시 load_dotenv(override=True) 로 .env 를 읽는데, 이 테스트들이 GEMINI_CLI_BINARY 를 monkeypatch 한 뒤 importlib.reload(config) 를 하면 reload 가 load_dotenv(override=True) 를 재실행하며 dev .env 의 agy 가 monkeypatch 값을 덮어씀(테스트 격리 결함). 수정: TestBinarySelection 의 _restore_gemini_default autouse fixture 에 monkeypatch.setattr('dotenv.load_dotenv', no-op) 추가 -&gt; reload 가 .env 를 다시 읽지 않아 monkeypatch 값 유지. monkeypatch 가 fixture teardown 이후 undo 되므로 teardown reload 동안에도 패치 유효(기본값 gemini 정상 복원). production config.py 의 override=True 는 봇 정책상 의도라 미변경. TestBinarySelection 10건 통과(4실패-&gt;0), 전체 421건 통과. Codex 교차검증 통과(발견 이슈 전부 Minor/Trivial).</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>테스트 스위트(test_gemini.py), CI/로컬 개발 신뢰성</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>v0.8.11</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>v0.8.12</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(watchdog): 크로스세션 워치독 중복 완화 - lockfile alive-check (v0.8.13)
!bot restart 한 번에 봇이 세션 수만큼(실측 4중) 중복 spawn 되던 회귀.
단일 인스턴스 mutex 이름이 Local\slack_multi_agent_watchdog 로 세션별
네임스페이스라, 예약작업 2개(SlackBotWatchdog=Interactive,
SlackBotWatchdogGuard=S4U 세션0)가 서로 다른 세션에서 띄운 워치독끼리
배제되지 않고 무기한 공존(실측 워치독 5개) -> 각자 restart 처리.

- watchdog.py acquire_lock(win32): mutex 획득 전에 .watchdog.lock 의 PID 를
  _is_pid_alive(OpenProcess, 세션 무관)로 확인, 살아있는 다른 워치독이 있으면
  exit(0). Local mutex 는 동일 세션 원자성용으로 유지.
- Global\ mutex 는 S4U Limited 에서 SeCreateGlobalPrivilege 부재 시 생성
  실패(fail-closed) 위험이라 회피.

알려진 한계(후속 LockFileEx 로 추적): 서로 다른 세션의 두 워치독이 stale
lockfile 상태로 동시 cold-start 하면 둘 다 통과하는 잔여 레이스. 정상상태는
단일 인스턴스로 수렴. 이미 떠 있는 세션0 스테일 프로세스는 관리자 권한 정리 필요.

신규 테스트 3건 + 기존 mutex 테스트 2건 tmp_path 결정론화. watchdog 20건 /
전체 424건 통과. Codex 교차검증 PASS(로직/무회귀/Global 회피 정당성).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7842,6 +7842,118 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>!bot restart 한 번에 봇이 세션 수만큼(4중) 중복 spawn (크로스세션 워치독 중복)</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>예약작업 2개(SlackBotWatchdog=Interactive, SlackBotWatchdogGuard=S4U 세션0)로 서로 다른 세션에 워치독이 각각 기동된 상태</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>1. 로그온 세션이 다른 워치독이 2개 이상 동시 가동(실측 5개: 세션0 4 + 대화형 1) 2. Slack 에서 !bot restart 1회 입력 3. 각 워치독이 명령을 독립 처리해 봇을 하나씩 spawn + '재시작 완료, Bot 시작됨(PID)' 메시지가 서로 다른 PID 로 4번 게시</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>원인: watchdog.py 단일 인스턴스 mutex 이름이 'Local\slack_multi_agent_watchdog' 로 세션별(per-logon-session) 네임스페이스라 세션이 다른 워치독끼리 배제하지 못하고 무기한 공존(+ mutex 도입 전 6월 스테일 워치독 누적). 수정: acquire_lock 의 win32 경로에서 mutex 획득 전에 .watchdog.lock 의 PID 를 _is_pid_alive(OpenProcess, 세션 무관)로 확인해 살아있는 다른 워치독이 있으면 exit(0). Local mutex 는 동일 세션 원자성용으로 유지. Global mutex 는 S4U Limited 에서 SeCreateGlobalPrivilege 부재 시 생성 실패(fail-closed)로 워치독이 아예 안 뜰 위험이라 회피. 신규 테스트 3건 + 기존 mutex 테스트 2건 결정론화, watchdog 20건/전체 424건 통과. Codex 교차검증 PASS(로직/무회귀/Global회피 정당성). 잔여 동시 cold-start 레이스는 알려진 한계로 후속 LockFileEx 하드닝(별도 이슈) 추적. 이미 떠 있는 세션0 스테일 프로세스는 관리자 권한으로 별도 정리 필요.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>watchdog.py 단일 인스턴스, !bot restart, 봇 중복 응답/토큰 낭비</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>v0.8.9</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>v0.8.13</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>워치독 크로스세션 단일 인스턴스 원자적 봉합 (LockFileEx)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>acquire_lock 의 크로스세션 배제를 lockfile alive-check(비원자적)에서 LockFileEx 커널 파일락(세션 무관, 특권 불필요, 프로세스 종료 시 OS 자동 해제)으로 보강해 동시 cold-start 레이스를 완전 봉합. PID 신원검증(생성시각/cmdline 대조)을 병행해 PID 재사용 오탐도 제거.</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>v0.8.13 의 lockfile alive-check 는 서로 다른 세션의 두 워치독이 stale lockfile 상태로 '동시에' cold-start 하면 둘 다 pre-check 를 통과하는 잔여 레이스가 있음(Codex Major). 정상상태는 단일 인스턴스로 수렴하나 원자적 보장은 아님.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>watchdog.py 단일 인스턴스</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>v0.8.13</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: v0.8.15 릴리즈 노트 + 이슈 로그(#128 agy #76 재검증·winpty 부적합 판정)
agy -p stdout 미출력 버그(upstream #76)에 대한 winpty 우회 대안을 실호출로
비교 검증. winpty 는 비-TTY subprocess 에서 'stdin is not a tty' 로 실행
불가(봇 부적합), agy 1.0.16 에서 #76 자체가 해소됨을 실측 확인. 현행 디스크
복구 방식 유지(무비용 안전망). 코드/테스트 무변경.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7957,6 +7957,62 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>agy `-p` stdout 버그(#76) 재검증 + winpty 우회 방식 부적합 판정</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>실호출 비교 테스트 3종을 봇과 동일 조건(stdin=DEVNULL, stdout=PIPE, AGY_CLI_DISABLE_AUTO_UPDATE=1)으로 수행: A) 순수 agy -p, B) winpty agy -p, C) 현재 디스크 transcript 복구(_recover_agy_response_retry 실코드).</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>agy 1.0.16(7/3 갱신)에서 upstream #76 이 해소되어 순수 agy -p 가 비-TTY 에서도 stdout 정상 출력(4회 100% 재현). winpty 방식은 winpty 자체가 stdin 이 tty 가 아니면 'stdin is not a tty' exit 1 로 실행 거부(DEVNULL/PIPE 동일, 우회 옵션 없음) -&gt; 봇 headless subprocess 에서 부적합. 현재 디스크 복구는 stdout 결손 시에만 발동하는 무비용 안전망이라 agy 회귀 대비 존치. 결론: winpty 교체 안 함, 현행 유지, 코드 무변경.</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>agents/gemini.py(agy 백엔드 경로), 봇 응답 수신</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>v0.8.14</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>v0.8.15</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Codex exec 실행 로그(exited -1073741502=0xC0000142 등) Slack 누출 필터 보강 (v0.8.16)
- agents/codex.py: _CODEX_EXEC_LOG_LINE 앵커드 정규식 신설(음수·소수 duration
  exit, MCP started/completed/failed/error, Output: 단독). 산문 오삭제 위험의
  기존 `exited 0/1 in` 서브스트링 리터럴 제거하고 정규식이 전담(^...$ 앵커).
- 근본원인 규명: 봇이 S4U 세션0(무데스크톱)에서 뜨면 Codex 셸/스킬 콘솔 자식이
  STATUS_DLL_INIT_FAILED 로 전멸(in-process MCP만 생존) → 무근거 답변. 활성 세션
  A/B 실측상 크래시 원인은 샌드박스 무관. 아키텍처 수정은 별도 이슈로 추적.
- 회귀 테스트 7건(TestExecLogLeak), 전체 432건 통과. Codex 교차검증 PASS(소수
  duration·MCP failed/error·기존 리터럴 제거 제안 3건 반영).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7976,7 +7976,6 @@
           <t>agy `-p` stdout 버그(#76) 재검증 + winpty 우회 방식 부적합 판정</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>실호출 비교 테스트 3종을 봇과 동일 조건(stdin=DEVNULL, stdout=PIPE, AGY_CLI_DISABLE_AUTO_UPDATE=1)으로 수행: A) 순수 agy -p, B) winpty agy -p, C) 현재 디스크 transcript 복구(_recover_agy_response_retry 실코드).</t>
@@ -8010,6 +8009,122 @@
       <c r="L129" t="inlineStr">
         <is>
           <t>Minor</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Codex exec 실행 로그(exited -1073741502 등)가 Slack 답변에 누출</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>봇이 S4U 세션0(무데스크톱)에서 구동돼 Codex 셸/스킬 자식이 0xC0000142 로 크래시하는 상태(별도 이슈)</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>1. 봇이 S4U 세션에서 가동 2. #ai-토론에 Codex 가 스킬/셸을 쓰게 되는 질문 입력(예: 'agy나 codex는 최상위 전역 메모리 기능이 없어?') 3. Codex 답변에 `Output:` 빈 블록, `exited -1073741502 in 31ms:`, `mcp: openaiDeveloperDocs/search_openai_docs (completed)` 조각이 그대로 노출됨</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>원인: _clean_codex_output 노이즈 필터가 `exited 0/1 in` 리터럴만 잡아 음수 exit code(-1073741502=0xC0000142 STATUS_DLL_INIT_FAILED)·`Output:` 단독·`mcp:` 라인을 못 걸렀음. 수정: `_CODEX_EXEC_LOG_LINE` 앵커드 정규식(음수·소수 duration, MCP started/completed/failed/error, Output:) 신설 후 정제 루프에 적용. 산문 오삭제 위험 있던 기존 `exited 0/1 in` 서브스트링 리터럴은 제거하고 정규식이 전담(^...$ 앵커라 '함수의 Output: 42'·'process exited 0 in my demo' 같은 본문은 보존). 회귀 테스트 7건 + 전체 432건 통과. Codex 교차검증 PASS(제안 3건 반영).</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>토론/리서치 모드 Codex 답변 표시(Slack), agents/codex.py</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>BE v0.8.15</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>BE v0.8.16</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>봇이 S4U 세션0(무데스크톱) 구동 시 Codex 셸/스킬 자식이 0xC0000142 로 전멸 → 무근거 답변</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>watchdog_guard(S4U, 세션0)가 단일 인스턴스 락을 먼저 잡아 봇을 세션0에서 spawn 한 상태</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>1. 봇이 S4U 가드 경로로 세션0에 기동 2. Codex 가 셸/스킬/웹 도구를 쓰려는 토론 질문 입력 3. Codex 의 모든 콘솔 자식 spawn 이 `exited -1073741502`(STATUS_DLL_INIT_FAILED)로 즉사, in-process MCP 만 성공 4. Codex 가 도구 없이 무근거로 답하며 'Claude 의견에 동의'로 얼버무림</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>원인: v0.8.1 에서 cmd 창 깜빡임 제거 목적으로 봇을 S4U 비대화형(세션0)으로 옮겼는데, 세션0 엔 데스크톱/윈도우스테이션이 없어 PowerShell·스킬 러너 등 콘솔 자식 프로세스가 DLL init 에 실패(0xC0000142). Interactive 세션에선 정상(활성 세션 A/B 실측: workspace-write·danger-full-access 둘 다 무크래시). 어느 워치독이 단일 락을 먼저 잡느냐로 세션이 갈림(watchdog_guard.start_watchdog 가 이기면 봇 트리가 세션0). 수정: 아키텍처 결정 대기(봇을 항상 데스크톱 세션에서 구동 vs 깜빡임 감수). 표면 로그 누출은 v0.8.16 필터로 봉합.</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>토론/리서치 모드 Codex 도구 사용(셸/스킬/웹), watchdog_guard.py·watchdog.py 세션, Codex 답변 품질</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>BE v0.8.1</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Major</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: 토론/리서치 Codex 셸 억제 지시(avoid_shell)로 S4U 세션0 크래시 회피 (v0.8.17, issue #131 Option 1)
봇이 S4U 세션0(무데스크톱)에서 뜨면 Codex 로컬 shell 도구(PowerShell spawn)가
0xC0000142(STATUS_DLL_INIT_FAILED)로 죽는다(issue #131). Slack 은 주로 토론/리서치
용도라 로컬 셸이 거의 불필요하고(MCP openaiDeveloperDocs + 지식으로 충분), cmd 창
깜빡임(v0.8.1~v0.8.2)을 되살리지 않는 Option 1 을 채택.

- agents/codex.py: _NO_SHELL_DIRECTIVE(로컬 셸 쓰지 말고 MCP/지식으로; read/MCP 허용)
  + CodexAgent(avoid_shell) + _maybe_prepend_directive(멱등). __init__ super() 호출.
- modes/debate.py, modes/research.py: Codex 메인+백업을 avoid_shell=True 로 생성.
  코딩 모드는 기본 False(셸 필요, 대화형 세션이면 정상).
- 실측(avoid_shell=True + 스레드 질문): 셸 시도/크래시 흔적 없이 MCP·지식 그라운딩
  답변, 미확인 항목은 단정 안 함. 회귀 5건, 전체 437건 통과.
- Codex 교차검증 반영: super().__init__() 추가 + 지시문 멱등 가드.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -8103,7 +8103,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>원인: v0.8.1 에서 cmd 창 깜빡임 제거 목적으로 봇을 S4U 비대화형(세션0)으로 옮겼는데, 세션0 엔 데스크톱/윈도우스테이션이 없어 PowerShell·스킬 러너 등 콘솔 자식 프로세스가 DLL init 에 실패(0xC0000142). Interactive 세션에선 정상(활성 세션 A/B 실측: workspace-write·danger-full-access 둘 다 무크래시). 어느 워치독이 단일 락을 먼저 잡느냐로 세션이 갈림(watchdog_guard.start_watchdog 가 이기면 봇 트리가 세션0). 수정: 아키텍처 결정 대기(봇을 항상 데스크톱 세션에서 구동 vs 깜빡임 감수). 표면 로그 누출은 v0.8.16 필터로 봉합.</t>
+          <t>원인: v0.8.1 에서 cmd 창 깜빡임 제거 목적으로 봇을 S4U 비대화형(세션0)으로 옮겼는데, 세션0 엔 데스크톱/윈도우스테이션이 없어 PowerShell·스킬 러너 등 콘솔 자식 프로세스가 DLL init 에 실패(0xC0000142). Interactive 세션에선 정상(활성 세션 A/B 실측: workspace-write·danger-full-access 둘 다 무크래시). 어느 워치독이 단일 락을 먼저 잡느냐로 세션이 갈림(watchdog_guard.start_watchdog 가 이기면 봇 트리가 세션0). 수정: 아키텍처 결정 대기(봇을 항상 데스크톱 세션에서 구동 vs 깜빡임 감수). 표면 로그 누출은 v0.8.16 필터로 봉합. [해결 v0.8.17 / Option 1: S4U(무깜빡임) 유지 + 토론/리서치 Codex 에 avoid_shell 지시 주입해 로컬 셸 시도 억제. Codex 는 openaiDeveloperDocs MCP·지식으로 그라운딩. 코딩 모드 셸 세션0 미동작은 드문 용도라 수용(완전 복구는 Option 2=대화형 상주, 깜빡임 부활).]</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -8116,10 +8116,14 @@
           <t>BE v0.8.1</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>BE v0.8.17</t>
+        </is>
+      </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">

</xml_diff>

<commit_message>
fix: 재기동 후 Codex 원격 MCP 일시적 503 누출/fatal 오탐 수정 (v0.8.18)
봇 재기동 직후 토론에서 원격 MCP openaiDeveloperDocs 초기화 중 일시적 HTTP 503 이
`<ISO8601>Z ERROR rmcp::transport::worker: ... HTTP 503 ...` tracing 로그로 답변에
누출되고, 그 'HTTP 503' 이 봇 _is_fatal_error 를 오탐시켜 유효 답변을 낸 Codex 가
백업(Gemini-B)으로 교체됐다(Slack thread 1783481931). 엔드포인트는 원격이라 세션
무관이며 조사 시점 정상(200) → 재기동 직후 일시적 blip.

- agents/codex.py: _CODEX_TRACING_LOG 정규식(ISO8601 타임스탬프+LEVEL target: 형식)
  으로 tracing 로그 라인 필터(누출 봉합). CodexAgent.ask_with_progress 가 base 의
  raw 기반 has_error 를 정제된 답변 기준으로 재판정(cleaned 비어있지 않고 timed_out
  아닐 때) → 일시적 MCP 오류로 벤치되지 않게. 진짜 API fatal 은 필터가 안 지워 유지.
- 회귀 6건(tracing 제거 3 + 재판정 3), 전체 443건 통과.
- Codex 교차검증 반영: 정규식 LEVEL target: 엄격화 + 넓은 rmcp:: substring 제거.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8132,6 +8132,66 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>재기동 후 Codex 가 원격 MCP 일시적 HTTP 503 로그를 답변에 누출 + fatal 오탐으로 백업 교체</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>봇이 재기동된 직후, 원격 MCP openaiDeveloperDocs(url=developers.openai.com/mcp) 엔드포인트가 일시적으로 503 반환</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>1. !bot restart 로 봇 재기동(세션0 유지) 2. 토론 질문 입력(예: 오늘 매수할만한 주식 추천) 3. Codex 답변 첫 줄에 `2026-...Z ERROR rmcp::transport::worker: worker quit with fatal: ... HTTP 503: upstream connect error ... when send initialized notification` 누출 4. 봇이 그 'HTTP 503' 을 Codex fatal 로 오탐 → 'Codex 오류 감지 → Gemini-B 대체 투입' 으로 교체(Codex 는 실제로 유효 추천을 냈음)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>원인: (1) v0.8.16 필터는 exec-log/Output:/mcp: 형식만 잡아 Rust tracing 로그(rmcp transport 오류)를 못 걸러 누출. (2) 봇은 progress 경로에서 정제 전 raw 로 _is_fatal_error 판정 → 로그의 'HTTP 503' 이 _FATAL_REGEX 에 걸려 has_error=True → 유효 답변인데도 백업 교체. openaiDeveloperDocs 는 원격이라 세션 무관, 503 은 재기동 직후 일시적 blip(조사 시점 엔드포인트 HTTP 200 정상). 수정: `_CODEX_TRACING_LOG` 정규식(ISO8601 타임스탬프+LEVEL target: 형식)으로 tracing 로그 라인 필터 + CodexAgent.ask_with_progress 가 has_error 를 정제된 답변 기준으로 재판정(cleaned 비어있지 않고 timed_out 아닐 때만; 진짜 API fatal 은 필터가 안 지우므로 유지). 회귀 6건 + 전체 443건 통과. Codex 교차검증 반영(정규식 엄격화, 넓은 rmcp:: substring 제거).</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>토론/리서치 모드 Codex 답변 표시 + 백업 교체 로직, agents/codex.py</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>BE v0.8.17</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>BE v0.8.18</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert "fix: 타임아웃 정책 전면 수정 - stale elapsed/숨은 배수/kill 사정거리 (v0.8.21)"
This reverts commit 18fb6a8fd9c445c33affaba13bdfdfcb73057d6b.
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8787,680 +8787,6 @@
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>142</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>코딩 수정 루프가 에이전트 실패 원문을 테스트 결과로 읽어 가짜 이슈를 만들고 코드를 산문으로 덮어씀 (재귀 오염)</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>코딩 모드 Phase 3(테스트 3병렬)에서 Claude 가 타임아웃하고 그 백업까지 실패한 상태</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>1. #ai-코딩 채널에 코딩 요청 2. Phase 3 에서 Claude 가 타임아웃 -&gt; "[Claude] 응답 대기 시간 초과 (574초 무응답)" 반환 3. 백업도 실패 4. 그 실패 문구가 all_tests 에 그대로 포함돼 Codex 이슈 판단 프롬프트로 전달됨 5. Codex 가 "이슈 있음: 타임아웃으로 테스트가 완료되지 않아 판단 불가" 를 이슈로 보고 6. 그 가짜 이슈로 Claude 에게 코드 수정 요청 -&gt; Claude 가 코드 대신 산문 반환 7. 산문이 current_code 가 되어 "[수정된 코드]" 로 게시되고 다음 라운드에 "기존 코드" 로 재투입</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>원인: BaseAgent 는 타임아웃/치명적 오류를 예외가 아니라 평범한 문자열로 반환하는데(agents/base.py:101,141,191,201), v0.8.19 는 이 실패 원문의 "게시"만 막고 "하류 전달"은 막지 않았다. modes/coding.py:871 이 실패한 슬롯의 문자열까지 all_tests 에 이어붙였고, 877 이 그걸 테스트 결과라며 Codex 에 넘겼다. 수정: (1) 실패한 Phase 3 슬롯을 None 으로 폐기하고 성공분만 all_tests 로 합침 (2) 테스트 결과 0건이면 이슈 판단 자체를 건너뜀 (3) Codex 이슈 판단이 실패하면 원문을 이슈로 삼지 않고 루프 중단 (4) Claude 수정 호출이 실패하면 current_code 를 덮어쓰지 않고 직전 코드 유지</t>
-        </is>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>코딩 모드 Phase 3 + 이슈 수정 루프 + 최종 보고서. 코드 산출물이 산문으로 대체되어 사용자에게 게시됨</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>BE v0.8.19</t>
-        </is>
-      </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L143" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Phase 1 주/백업 이중 실패 시 실패 문구가 claude_code 가 되어 그대로 리뷰/테스트됨</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Phase 1 에서 Claude 와 그 백업이 모두 실패(타임아웃/세션 한도)한 상태</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>1. 코딩 요청 2. Phase 1 Claude 타임아웃 -&gt; 백업 투입 -&gt; 백업도 세션 한도로 실패 3. _ask_with_backup 이 "[Claude] 응답을 받지 못했습니다 (백업 ... 도 실패)." 를 반환 4. 이 문구가 claude_code 로 Phase 2 리뷰 프롬프트와 Phase 3 테스트 프롬프트에 "코드" 로 삽입됨. 백업이 아예 없는 경우엔 실패 원문이 그대로 반환돼 답변으로 게시까지 됨</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>원인: modes/coding.py 의 Phase 1 호출부(_start_inner, followup 재개)가 _ask_with_backup 반환값의 성공 여부(needs_replacement)를 확인하지 않고 무조건 Phase 2/3 로 넘겼다. 또한 _ask_with_backup 은 백업 풀이 소진되면 실패 원문을 그대로 돌려줬다. 수정: Phase 1 실패 시 "코드 생성 실패 -&gt; 리뷰/테스트 단계 중단" 을 고지하고 후속 단계 진입을 차단. _ask_with_backup 은 백업이 없어도 실패 원문 대신 정제 문구를 반환하고 needs_replacement 로 실패를 알림</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>코딩 모드 Phase 1 -&gt; Phase 2/3 전이, 백업 풀 소진 경로</t>
-        </is>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>BE v0.8.19</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>144</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>병렬 모드에서 백업이 없는 실패 에이전트의 응답 원문이 최종 요약 프롬프트로 유입</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>코딩 병렬 모드에서 한 에이전트가 실패하고 그 백업이 없는 상태</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>1. 코딩 병렬 모드 실행 2. Claude 타임아웃, 백업 풀 소진 3. modes/coding.py:669-670 이 실패 원문을 final_responses 에 그대로 append 4. 678-679 가 그걸 "[Claude 결과]" 로 요약 프롬프트에 삽입 -&gt; Codex 가 타임아웃 문구를 작업 결과로 읽고 요약</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>원인: 백업이 존재할 때만 continue 로 빠져나가고, 백업이 없으면 실패한 에이전트와 그 실패 원문이 그대로 final_agents/final_responses 에 담겼다. 수정: 백업이 없거나 백업까지 실패하면 결과 없이 제외하고 사유를 고지. 전원 실패면 빈 요약을 요청하지 않고 중단</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>코딩 병렬 모드 최종 보고서</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>BE v0.8.19</t>
-        </is>
-      </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>최종 보고서 생성이 실패하면 그 실패 원문이 "최종 보고서" 로 방송됨</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>최종 보고서 작성 단계에서 Codex 가 타임아웃/오류로 실패한 상태</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>1. 코딩 모드 실행 2. 마지막 보고서 생성 호출에서 Codex 타임아웃 3. 반환된 "[Codex] 응답 시간 초과 (300초)" 가 그대로 "📋 최종 보고서 (Codex)" 로 broadcast 됨 (병렬 모드도 동일)</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>원인: 보고서 호출 결과의 needs_replacement 를 확인하지 않고 무조건 방송했다. 수정: 실패 시 방송하지 않고 "최종 보고서 생성 실패" 고지로 대체. 아울러 None(호출 실패)과 ""(내용 없는 정상 응답)을 구분하는 _test_summary() 를 도입해 보고서가 둘을 혼동하지 않게 함</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>코딩 모드/병렬 모드 최종 보고서 방송</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>BE v0.8.19</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>146</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>타임아웃 메시지가 실제보다 60초 적은 "574초" 로 표기되고 한도(600초)도 초과</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>코딩 모드에서 Claude 가 도구 호출 중 60초 이상 무응답인 상태</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>1. 코딩 모드 실행 2. Claude 가 스트리밍 중 장시간 무응답 3. 전체 한도 600초를 넘겨 종료되는데 Slack 에는 "[Claude] 응답 대기 시간 초과 (574초)" 로 게시됨 (실제 경과는 634초)</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>원인: agents/claude.py(및 동형인 gemini.py) 읽기 루프가 elapsed 를 루프 진입 시점에 재고, readline 을 고정 60초 기다린 뒤 그 stale 값을 메시지에 찍었다. 한도 검사도 루프 진입 시점에만 해서 readline_timeout(60초) 만큼 한도를 넘겼다(실효 상한 660초). 수정: readline 대기를 min(STREAM_IDLE_TIMEOUT, 남은 예산) 으로 자르고, 보고 직전 elapsed 를 재측정. 메시지에 한도를 병기(응답 시간 초과 (634초 / 한도 600초)). start_time 도 spawn 전으로 옮겨 spawn/stdin drain 시간을 예산에 포함(Codex 지적 반영)</t>
-        </is>
-      </c>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>코딩/토론/리서치 전 모드의 스트리밍 타임아웃 메시지 및 실제 상한</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>147</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>같은 timeout 인자가 에이전트마다 다른 예산을 의미 (Codex 300초 vs Claude 660초)</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>없음</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>1. 코딩 모드에서 timeout=CLI_TIMEOUT_CODING(300) 을 모든 에이전트에 동일하게 전달 2. 실제로는 base(Codex)=300초, Claude=600(+60)초, Gemini=600초/가드 750초로 제각각 3. 한 실행에 "[Claude] 응답 시간 초과 (300초)" 와 "(574초)" 가 동시에 찍힘</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>원인: 스트리밍 구현이 내부에서 timeout 을 조용히 t*2 로 늘렸고 base 구현은 안 늘렸다. 수정: 숨은 배수 제거. timeout 이 곧 예산. 모드별 예산을 상수로 승격 (CLI_TIMEOUT 180-&gt;360, CLI_TIMEOUT_CODING 300-&gt;600, CLI_TIMEOUT_RESEARCH 180 신설). 실효 예산은 의도적으로 조정됨: 코딩 Claude 660-&gt;600(축소), 코딩 Codex 300-&gt;600(확대). Codex 확대는 의도 - 예전엔 절반 예산이라 정상 장시간 작업 중 혼자 먼저 타임아웃 나 불필요하게 백업 교체됐다. 토론 라운드 체감 상한은 420-&gt;360초로 오히려 감소</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>전 모드 에이전트 호출 예산, 백업 교체 빈도</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>148</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>한 에이전트의 타임아웃이 병렬 실행 중인 형제 에이전트의 프로세스까지 kill</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>여러 에이전트가 asyncio.gather 로 병렬 실행 중 (코딩 Phase 3, 리서치 분담 조사)</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>1. 코딩 Phase 3 에서 Codex/Claude/Gemini 가 같은 thread_ts 로 병렬 실행 2. 그 중 하나가 타임아웃 3. _kill_registered_processes() 가 thread_ts 에 등록된 모든 프로세스를 죽여 멀쩡히 돌던 나머지 에이전트도 동반 실패 4. 테스트 결과 0건 -&gt; Codex 가짜 이슈 -&gt; 수정 루프 헛돎</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>원인: cancel.active_processes 가 thread_ts 단위 레지스트리인데 타임아웃 정리가 그걸 그대로 순회해 전부 죽였다. 모든 에이전트는 같은 _current_thread_ts 를 공유한다. 게다가 리서치는 하위질문을 라운드로빈 배정하므로 같은 인스턴스가 동시에 2건을 맡기도 한다(4문항/3에이전트). 수정: contextvars.ContextVar + AgentBase._call_scope() 로 kill 사정거리를 호출 단위로 축소. 사용자 취소(/cancel)는 기존대로 스레드 전체 kill 유지</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>코딩 Phase 3, 리서치 분담 조사, 토론 라운드 (병렬 실행 전 구간)</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>149</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Claude 스트리밍에 외부 가드가 없어 읽기 루프 밖 hang 이 영구 대기</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>stdin drain 이 막히거나 proc.wait() 이 복귀하지 않는 상태</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>1. Claude CLI 가 stdin 을 읽지 않아 파이프 버퍼가 참 2. await proc.stdin.drain() 이 영구 블록 3. 읽기 루프에 진입조차 못 해 내부 데드라인 검사가 발동하지 않음 4. 봇 정지</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>원인: 내부 데드라인은 읽기 루프 안에서만 검사된다. 루프 밖 await(stdin drain, proc.wait)은 그 검사에 도달하지 못한다. Gemini 는 v0.7.3.2 에서 외부 가드를 받았지만 Claude 는 무방비였다. 수정: base.ask_with_progress 가 _stream_once 를 t*STREAM_GUARD_FACTOR(1.25) 로 감싼다. Claude 는 _stream_once 만 오버라이드하도록 정리했고 Codex 는 super() 위임이라 자동 적용. 상한은 정상 t, 병리적 hang 시 t*1.25</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>Claude/Codex 스트리밍 호출 (코딩 전 Phase, 토론 라운드)</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>외부 가드 취소 시 살아있는 CLI 를 죽이기 전에 부산물을 지워 임시 폴더에 파일 누수</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>외부 가드가 발동해 _stream_once 코루틴이 cancel 되는 상태</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>1. 외부 가드(asyncio.wait_for) 타임아웃 2. wait_for 가 내부 Task 를 cancel 하고 그 Task 의 finally 가 먼저 완료됨 3. 그 finally 가 아직 살아있는 CLI 의 -o &lt;tmp&gt;.last.md 부산물과 프롬프트 파일을 삭제 4. 그 뒤에야 호출부 except 가 프로세스를 kill 5. 삭제와 kill 사이에 살아있는 writer 가 파일을 다시 써서 임시 폴더에 남음</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>원인: 정리 순서가 (파일 삭제 -&gt; 프로세스 kill) 이었다. asyncio.wait_for 는 내부 Task 의 finally 가 끝난 뒤에야 호출부로 제어를 넘기므로, 파일 정리 시점에 CLI 가 아직 살아있다. 수정: _kill_if_alive() 를 파일 정리 앞에 배치해 writer 를 먼저 죽인다(kill_process_tree 는 동기 함수라 cancel 중인 finally 안에서도 안전 - 여기서 await 하면 CancelledError 가 재발생해 정리가 중단된다). Codex 교차검증 지적 반영</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>CodexAgent 의 -o 최종 메시지 파일, 전 에이전트의 프롬프트 임시 파일</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>151</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>bug</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>코딩 모드 백업 에이전트가 primary 보다 짧은 예산으로 호출됨</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>primary 에이전트가 타임아웃/오류로 백업 교체가 트리거된 상태</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>1. 코딩 모드에서 primary 가 코딩 예산(600초)을 다 쓰고 타임아웃 2. _ask_with_backup 이 backup.ask(prompt) 를 timeout 인자 없이 호출 3. 백업은 기본 예산(CLI_TIMEOUT)만 받아 primary 보다 짧은 시간 안에 끝내야 함</t>
-        </is>
-      </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>원인: modes/coding.py 의 백업 호출만 timeout 인자를 빠뜨렸다(다른 백업 경로는 CLI_TIMEOUT_CODING 을 넘긴다). primary 가 코딩 예산으로도 못 끝낸 일을 더 짧은 예산으로 시키는 꼴이라 이중 실패(백업도 실패) 확률만 올라간다. 수정: timeout=CLI_TIMEOUT_CODING 명시. 재시도 정책 점검 결과 타임아웃 자체는 재시도하지 않고(같은 예산 재실행은 실패 시간만 2배) 곧바로 백업 교체하되, 백업은 primary 와 같은 예산을 받는 것으로 확정</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>코딩 모드 백업 교체 경로</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>BE v0.8.20</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>enhancement</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>에이전트 상태 플래그(timed_out/has_error/last_usage)가 인스턴스 공유라 병렬 호출에 취약</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>리서치가 같은 에이전트 인스턴스를 병렬 호출하는데(라운드로빈 배정: 4문항/3에이전트) timed_out/has_error/last_usage 는 인스턴스 속성이다. 호출별 상태 객체로 분리하거나 호출 결과에 상태를 함께 반환해 공유 플래그 판정을 제거해야 한다.</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>v0.8.21 에서 프로세스 kill 사정거리는 호출 단위로 좁혔으나 상태 플래그는 여전히 인스턴스 공유다. 현재 호출부는 ask() 반환 직후 await 없이 곧바로 플래그를 읽으므로(이벤트 루프가 그 사이에 다른 코루틴을 끼워넣지 못함) 실제 트리거는 확인되지 않았다. 다만 호출부에 await 가 하나만 끼어들면 곧바로 오판(한 호출의 실패가 다른 호출의 백업 교체를 유발)으로 이어지는 구조적 취약점이라 선제 정리가 필요하다. Codex 교차검증 지적 반영</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>리서치 분담 조사, 향후 동일 인스턴스 병렬 호출을 추가하는 모든 경로</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>BE v0.8.21</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>진행중</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(log): 조인 키가 빈 행 2건에 Linear 이슈를 만들고 키를 채운다 (SYM-11, SYM-12)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FigcsmP85LkasfoHXsHcwK
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -422,7 +422,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V150"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -7533,6 +7533,16 @@
           <t>bug</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
           <t>v0.7.3.2 핫픽스 누락: _run_progress_once L293 _gemini_concurrency 잔존 + cancel cleanup 부재</t>
@@ -7576,6 +7586,11 @@
           <t>완료</t>
         </is>
       </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>SYM-11</t>
+        </is>
+      </c>
       <c r="V99" t="inlineStr">
         <is>
           <t>Block</t>
@@ -11127,6 +11142,16 @@
           <t>bug</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
       <c r="F149" t="inlineStr">
         <is>
           <t>agy 콘솔 창 깜빡임 (이슈 #112 wontfix 재조사 후 해결)</t>
@@ -11169,6 +11194,11 @@
       <c r="T149" t="inlineStr">
         <is>
           <t>완료</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>SYM-12</t>
         </is>
       </c>
       <c r="V149" t="inlineStr">

</xml_diff>